<commit_message>
docs: v5.11 decision table on confirmed Whitefields quantities; CS roof on footprint basis
Whitefields: 3,740 m2 GIA, 2,210 m2 footprint, 8,000 m2 site (owner,
3 Oct). Demolition moves from Hold to Change (Std 130 -> 100); asbestos
kept at 25 (matches Mace's pre-tender allowance). Roof 2.5a: CS is 182
per m2 footprint, not 313 (re-covered 699 of 1,199 m2), so the proposal
becomes 120 / 190 / 400, High provisional until the Claycroft roof
package is checked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QB69m6diVrBfvTZaLwAazz
</commit_message>
<xml_diff>
--- a/docs/nrm1-v5.11-rate-decisions.xlsx
+++ b/docs/nrm1-v5.11-rate-decisions.xlsx
@@ -84,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8E8EE"/>
+        <fgColor rgb="00E3EFE3"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,12 +94,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E3EFE3"/>
+        <fgColor rgb="00FCE9C8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE9C8"/>
+        <fgColor rgb="00E8E8EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,19 +165,19 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -655,7 +655,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>WF = Whitefields demolition — Total Reclaims contract 2026 (× 1.014). GIA ASSUMED at 3,000 m² (footprint × 1.5) — please confirm. PR #35.</t>
+          <t>WF = Whitefields demolition — Total Reclaims contract 2026 (× 1.014). Quantities confirmed by you on 3 Oct: 17 blocks, 3,740 m² GIA, 2,210 m² footprint, 8,000 m² site. PR #35.</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>• Demolition rates look high against Whitefields, but its GIA is assumed — hold until confirmed.</t>
+          <t>• Demolition is over-priced against Whitefields (confirmed quantities): £73 vs £130 per m² demolished. Asbestos kept — the tender came in at a third of Mace's pre-tender allowance.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>• Confirm the Whitefields GIA (drives asbestos and demolition per m²).</t>
+          <t>• Check the Claycroft roof package (about £2.70m in the G4 contract, 5,747 m² roof plan) before the roof High rate is set.</t>
         </is>
       </c>
     </row>
@@ -956,13 +956,13 @@
       <c r="M5" s="7" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>£10.1 (5 bids £10–£53, median £15.8)</t>
+          <t>£8.1 (5 bids £8.1–£42.5, median £12.7; Mace pre-tender £24.5)</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr"/>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>Hold</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="Q5" s="8" t="n"/>
@@ -973,7 +973,7 @@
       <c r="T5" s="10" t="n"/>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>One demolition job and its GIA is assumed. Asbestos depends on the survey. Keep £25 until the GIA is confirmed and a second project is in.</t>
+          <t>Mace's pre-tender allowance (£24.5) matches the workbook; the tender came in at a third of it. At Stage 0–1 the extent of asbestos is unknown, so keep £25 until a second project shows the same.</t>
         </is>
       </c>
       <c r="V5" s="11" t="inlineStr"/>
@@ -1018,24 +1018,26 @@
       <c r="M6" s="7" t="inlineStr"/>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>£91 incl. disconnections (core demolition £43; 5 bids £43–£87)</t>
+          <t>£73 incl. disconnections £39 (core demolition £34; 5 bids £34–£70, median £46)</t>
         </is>
       </c>
       <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr">
-        <is>
-          <t>Hold</t>
+      <c r="P6" s="12" t="inlineStr">
+        <is>
+          <t>Change</t>
         </is>
       </c>
       <c r="Q6" s="8" t="n"/>
-      <c r="R6" s="8" t="n">
-        <v>130</v>
+      <c r="R6" s="13" t="n">
+        <v>100</v>
       </c>
       <c r="S6" s="8" t="n"/>
-      <c r="T6" s="10" t="n"/>
+      <c r="T6" s="10" t="n">
+        <v>-0.2307692307692307</v>
+      </c>
       <c r="U6" s="7" t="inlineStr">
         <is>
-          <t>Points to about £100, but per-m² depends on the assumed 3,000 m² GIA. If you confirm it, change Std to £100.</t>
+          <t>On your confirmed 3,740 m² GIA the contract is £73 per m² demolished, 44% under £130. Whitefields is simple two-storey masonry, so £100 (not £73) leaves room for framed or taller buildings. One rate for every spec level, as now.</t>
         </is>
       </c>
       <c r="V6" s="11" t="inlineStr"/>
@@ -1088,7 +1090,7 @@
           <t>£51</t>
         </is>
       </c>
-      <c r="P7" s="12" t="inlineStr">
+      <c r="P7" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1146,11 +1148,11 @@
       <c r="M8" s="7" t="inlineStr"/>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>£40 (£49 with pending changes)</t>
+          <t>£36 (£44 with pending changes); £315 per m of main</t>
         </is>
       </c>
       <c r="O8" s="7" t="inlineStr"/>
-      <c r="P8" s="12" t="inlineStr">
+      <c r="P8" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1211,35 +1213,35 @@
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>£313 flat warm-roof overlay (bids £288–£338)</t>
+          <t>£182 per m² footprint (£313 per m² re-covered × 699 / 1,199 m²) — flat warm-roof overlay</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr"/>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>£517 metal over-roof (£601 out-turn); scaffold extra</t>
-        </is>
-      </c>
-      <c r="P9" s="13" t="inlineStr">
+          <t>£517 per m² roof plan, metal over-roof — TO CHECK (≈ £2.70m package)</t>
+        </is>
+      </c>
+      <c r="P9" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="Q9" s="14" t="n">
-        <v>160</v>
-      </c>
-      <c r="R9" s="14" t="n">
-        <v>300</v>
-      </c>
-      <c r="S9" s="14" t="n">
-        <v>520</v>
+      <c r="Q9" s="13" t="n">
+        <v>120</v>
+      </c>
+      <c r="R9" s="13" t="n">
+        <v>190</v>
+      </c>
+      <c r="S9" s="13" t="n">
+        <v>400</v>
       </c>
       <c r="T9" s="10" t="n">
-        <v>1.727272727272727</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>Both projects are 2.8–4.7× today's Std. Std £300 = CS flat roof; High £520 = Claycroft over-roof. Refurb Std then equals New build Std (£300), which is realistic for a full re-roof. New build not changed.</t>
+          <t>The app prices the roof on the full footprint, so CS is £182 on that basis (it re-covered only 699 of 1,199 m²). Std £190 = CS. High £400 is provisional until the Claycroft roof package is checked. New build not changed.</t>
         </is>
       </c>
       <c r="V9" s="11" t="inlineStr"/>
@@ -1292,7 +1294,7 @@
       </c>
       <c r="N10" s="7" t="inlineStr"/>
       <c r="O10" s="7" t="inlineStr"/>
-      <c r="P10" s="12" t="inlineStr">
+      <c r="P10" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1362,7 +1364,7 @@
       </c>
       <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="7" t="inlineStr"/>
-      <c r="P11" s="13" t="inlineStr">
+      <c r="P11" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
@@ -1373,7 +1375,7 @@
       <c r="R11" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="S11" s="14" t="n">
+      <c r="S11" s="13" t="n">
         <v>210</v>
       </c>
       <c r="T11" s="10" t="n"/>
@@ -1436,7 +1438,7 @@
           <t>£96 out-turn (£22 provisional sum in contract)</t>
         </is>
       </c>
-      <c r="P12" s="13" t="inlineStr">
+      <c r="P12" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
@@ -1447,7 +1449,7 @@
       <c r="R12" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="S12" s="14" t="n">
+      <c r="S12" s="13" t="n">
         <v>95</v>
       </c>
       <c r="T12" s="10" t="n"/>
@@ -1510,7 +1512,7 @@
           <t>£99 incl. ceiling/door painting and PVC cladding</t>
         </is>
       </c>
-      <c r="P13" s="12" t="inlineStr">
+      <c r="P13" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1584,7 +1586,7 @@
           <t>£38</t>
         </is>
       </c>
-      <c r="P14" s="12" t="inlineStr">
+      <c r="P14" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1658,7 +1660,7 @@
           <t>£70 full replacement, fire-line board</t>
         </is>
       </c>
-      <c r="P15" s="12" t="inlineStr">
+      <c r="P15" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1732,7 +1734,7 @@
           <t>£3,869 IPS + vanity</t>
         </is>
       </c>
-      <c r="P16" s="12" t="inlineStr">
+      <c r="P16" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1802,7 +1804,7 @@
           <t>£64 (mostly bathroom boxings)</t>
         </is>
       </c>
-      <c r="P17" s="12" t="inlineStr">
+      <c r="P17" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -1878,18 +1880,18 @@
       </c>
       <c r="N18" s="7" t="inlineStr"/>
       <c r="O18" s="7" t="inlineStr"/>
-      <c r="P18" s="13" t="inlineStr">
+      <c r="P18" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="Q18" s="14" t="n">
+      <c r="Q18" s="13" t="n">
         <v>110</v>
       </c>
-      <c r="R18" s="14" t="n">
+      <c r="R18" s="13" t="n">
         <v>190</v>
       </c>
-      <c r="S18" s="14" t="n">
+      <c r="S18" s="13" t="n">
         <v>260</v>
       </c>
       <c r="T18" s="10" t="n">
@@ -1950,7 +1952,7 @@
           <t>£39 partial replacement</t>
         </is>
       </c>
-      <c r="P19" s="12" t="inlineStr">
+      <c r="P19" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2026,7 +2028,7 @@
       <c r="M20" s="7" t="inlineStr"/>
       <c r="N20" s="7" t="inlineStr"/>
       <c r="O20" s="7" t="inlineStr"/>
-      <c r="P20" s="9" t="inlineStr">
+      <c r="P20" s="14" t="inlineStr">
         <is>
           <t>Reject #31</t>
         </is>
@@ -2102,7 +2104,7 @@
           <t>£92 out-turn incl. new ductwork and roof fans</t>
         </is>
       </c>
-      <c r="P21" s="12" t="inlineStr">
+      <c r="P21" s="9" t="inlineStr">
         <is>
           <t>Take #31</t>
         </is>
@@ -2178,7 +2180,7 @@
           <t>£28 incl. fire dampers</t>
         </is>
       </c>
-      <c r="P22" s="12" t="inlineStr">
+      <c r="P22" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2254,7 +2256,7 @@
           <t>£4.3 (interfaces only — not comparable)</t>
         </is>
       </c>
-      <c r="P23" s="12" t="inlineStr">
+      <c r="P23" s="9" t="inlineStr">
         <is>
           <t>Take #31</t>
         </is>
@@ -2330,7 +2332,7 @@
           <t>£158</t>
         </is>
       </c>
-      <c r="P24" s="12" t="inlineStr">
+      <c r="P24" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2410,18 +2412,18 @@
           <t>£113 incl. emergency and external</t>
         </is>
       </c>
-      <c r="P25" s="13" t="inlineStr">
+      <c r="P25" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="Q25" s="14" t="n">
+      <c r="Q25" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="R25" s="14" t="n">
+      <c r="R25" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="S25" s="14" t="n">
+      <c r="S25" s="13" t="n">
         <v>85</v>
       </c>
       <c r="T25" s="10" t="n">
@@ -2492,18 +2494,18 @@
           <t>£65 new system throughout</t>
         </is>
       </c>
-      <c r="P26" s="13" t="inlineStr">
+      <c r="P26" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="Q26" s="14" t="n">
+      <c r="Q26" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="R26" s="14" t="n">
+      <c r="R26" s="13" t="n">
         <v>20</v>
       </c>
-      <c r="S26" s="14" t="n">
+      <c r="S26" s="13" t="n">
         <v>65</v>
       </c>
       <c r="T26" s="10" t="n">
@@ -2568,7 +2570,7 @@
           <t>£19 data only</t>
         </is>
       </c>
-      <c r="P27" s="12" t="inlineStr">
+      <c r="P27" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2644,18 +2646,18 @@
           <t>£112,850 replacement incl. design</t>
         </is>
       </c>
-      <c r="P28" s="13" t="inlineStr">
+      <c r="P28" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
       </c>
-      <c r="Q28" s="14" t="n">
+      <c r="Q28" s="13" t="n">
         <v>60000</v>
       </c>
-      <c r="R28" s="14" t="n">
+      <c r="R28" s="13" t="n">
         <v>100000</v>
       </c>
-      <c r="S28" s="14" t="n">
+      <c r="S28" s="13" t="n">
         <v>130000</v>
       </c>
       <c r="T28" s="10" t="n">
@@ -2716,7 +2718,7 @@
       </c>
       <c r="N29" s="7" t="inlineStr"/>
       <c r="O29" s="7" t="inlineStr"/>
-      <c r="P29" s="12" t="inlineStr">
+      <c r="P29" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2790,7 +2792,7 @@
           <t>£11 (more BWIC inside M&amp;E lines)</t>
         </is>
       </c>
-      <c r="P30" s="12" t="inlineStr">
+      <c r="P30" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2860,7 +2862,7 @@
       </c>
       <c r="N31" s="7" t="inlineStr"/>
       <c r="O31" s="7" t="inlineStr"/>
-      <c r="P31" s="12" t="inlineStr">
+      <c r="P31" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2930,7 +2932,7 @@
           <t>£164 defects found in out-turn</t>
         </is>
       </c>
-      <c r="P32" s="12" t="inlineStr">
+      <c r="P32" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -2996,11 +2998,11 @@
       <c r="M33" s="7" t="inlineStr"/>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>£2.2 topsoil and seed only</t>
+          <t>£2.1 topsoil and seed only</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr"/>
-      <c r="P33" s="12" t="inlineStr">
+      <c r="P33" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -5695,7 +5697,7 @@
           <t>L 7–11% (median ~9%, occupied flats). CC 11.3% (Tier 1, occupied, £21m). WF 16.8% incl. £39k hoarding (£0.5m demolition). CS not recorded.</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
@@ -5734,7 +5736,7 @@
           <t>L 7.5% median (6–10%) at £1–5m. WF 15% at &lt; £1m. CC 2.2% SCAPE fee + 2.1% design + 2.8% risk = 7.1% at &gt; £5m.</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Keep</t>
         </is>
@@ -5773,7 +5775,7 @@
           <t>CS: everything above construction (fees, surveys, Estates) = 14.7%. WF 28% + 4% Estates — ecology and environmental monitoring £67k on a £0.5m demolition.</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>Hold</t>
         </is>
@@ -5812,7 +5814,7 @@
           <t>CC +33% out-turn against a 21.5% client allowance (defects £2.65m, fire stopping £2.63m, M&amp;E £1.40m). CS +3.4%. WF holds 65% risk, 1% drawn so far.</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>Change</t>
         </is>
@@ -5916,7 +5918,7 @@
           <t>CS £42/m² GIFA (bids £35–£49). CC £33/m² GIA (£99/m² roof plan).</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Add</t>
         </is>
@@ -5945,7 +5947,7 @@
           <t>CS out-turn £781/m² construction for an envelope + heat-pump retrofit; band is £800–1,800/m².</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Hold</t>
         </is>
@@ -5974,7 +5976,7 @@
           <t>Your decision on 29 Sept.</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Take #31</t>
         </is>
@@ -6003,7 +6005,7 @@
           <t>Mid sat outside its own 0.93–1.00 range.</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Take #31</t>
         </is>
@@ -6032,7 +6034,7 @@
           <t>CC: £350k provisional sum became £2.63m incl. compartment-wall heads.</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Add</t>
         </is>

</xml_diff>